<commit_message>
Fix excel closing bug
</commit_message>
<xml_diff>
--- a/src/modeling/driver_pred_list.xlsx
+++ b/src/modeling/driver_pred_list.xlsx
@@ -10,6 +10,7 @@
     <sheet name="list" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="drivers" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="teams" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="races" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,11 +416,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -438,6 +440,11 @@
           <t>team</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>grand_prix</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -453,6 +460,11 @@
           <t>Alpine</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -770,12 +782,15 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="B2 B3 B4 B5 B6 B7 B8 B9 B10 B11 B12 B13 B14 B15 B16 B17 B18 B19 B20 B21 B22 B23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>drivers!$A$1:$A$43</formula1>
     </dataValidation>
     <dataValidation sqref="C2 C3 C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>teams!$A$1:$A$17</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2 D3 D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>races!$A$1:$A$34</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1228,4 +1243,256 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>70th Anniversary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Abu Dhabi</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Azerbaijan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bahrain</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Eifel</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Emilia-Romagna</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Great Britain</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Las Vegas</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Miami</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Russia</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Sakhir</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Saudi Arabia</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Styria</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Tuscany</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>